<commit_message>
Updates after June meeting.
</commit_message>
<xml_diff>
--- a/Subgroups/ASX/Proposed Extension Working Materials/ASX Standard Definition WBS.xlsx
+++ b/Subgroups/ASX/Proposed Extension Working Materials/ASX Standard Definition WBS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hosang\Documents\6 - SISO\C2SIMDocs\ASX\C2SIMArtifacts\Subgroups\ASX\Proposed Extension Working Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E1BCF4-6C96-4977-AD6F-E27A37E5CB23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A76172C-FB18-4B52-8813-4F1C23A3AD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
   <si>
     <t>1</t>
   </si>
@@ -200,6 +200,9 @@
   </si>
   <si>
     <t>Michael</t>
+  </si>
+  <si>
+    <t>Generate schema from OWL model</t>
   </si>
 </sst>
 </file>
@@ -665,7 +668,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>